<commit_message>
excel template and imprt data updated 16-02-2025
</commit_message>
<xml_diff>
--- a/sourceEnq/Template-Ar.xlsx
+++ b/sourceEnq/Template-Ar.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27726"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Houda\Documents\SDL3\sourceEnq\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\develepement\SDL3\sourceEnq\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F1E7A9-75A3-47C3-B7B0-BC6A99A389FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Arabe" sheetId="2" r:id="rId1"/>
@@ -33,14 +32,6 @@
     <t>العدد</t>
   </si>
   <si>
-    <t>رقـــم 
-الملــــــف</t>
-  </si>
-  <si>
-    <t>تاريــــخ 
-الايـــداع</t>
-  </si>
-  <si>
     <t>اللقــــب</t>
   </si>
   <si>
@@ -53,103 +44,15 @@
     <t>تاريخ الميلاد</t>
   </si>
   <si>
-    <t>رقـم عقد الميـــــلاد</t>
-  </si>
-  <si>
-    <t>بلــدية الميــــلاد</t>
-  </si>
-  <si>
     <t>الحالة العائلية</t>
   </si>
   <si>
-    <t>اســــــــم الاب</t>
-  </si>
-  <si>
-    <t>لقــــــب الام</t>
-  </si>
-  <si>
-    <t>اســــم الام</t>
-  </si>
-  <si>
     <t>العنـــــــــــــــــــــــــــــــــــــــــوان</t>
   </si>
   <si>
-    <t>لقـــب الــزوج(ة)</t>
-  </si>
-  <si>
-    <t>تاريـخ ميـــلاد
- الـــــــــزوج (ة)</t>
-  </si>
-  <si>
-    <t>رقم عقد ميلاد الـــزوج(ة)</t>
-  </si>
-  <si>
-    <t>بلـــدية ميــــــلاد الـــــــــــــزوج(ة)</t>
-  </si>
-  <si>
-    <t>اســم أم الـــــزوج (ة)</t>
-  </si>
-  <si>
-    <t>لقـــب أم الــزوج(ة)</t>
-  </si>
-  <si>
     <t>المجموع</t>
   </si>
   <si>
-    <t>الملاحظـــــــــــــــــــــــــــة</t>
-  </si>
-  <si>
-    <r>
-      <t>اســــم 
-الـــزوج(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="20"/>
-        <color indexed="10"/>
-        <rFont val="Mohammad Bold Normal"/>
-        <charset val="178"/>
-      </rPr>
-      <t>ة</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="20"/>
-        <color indexed="8"/>
-        <rFont val="Mohammad Bold Normal"/>
-        <charset val="178"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>اســـــــم أب الـــــزوج(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="20"/>
-        <color indexed="10"/>
-        <rFont val="Mohammad Bold Normal"/>
-        <charset val="178"/>
-      </rPr>
-      <t>ة</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="20"/>
-        <color indexed="8"/>
-        <rFont val="Mohammad Bold Normal"/>
-        <charset val="178"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
     <t>عدد الزوجات</t>
   </si>
   <si>
@@ -172,16 +75,64 @@
   </si>
   <si>
     <t>رقم التعريف الوطني</t>
+  </si>
+  <si>
+    <t>رقم الملف</t>
+  </si>
+  <si>
+    <t>تاريخ الايداع</t>
+  </si>
+  <si>
+    <t>رقم عقد الميلاد</t>
+  </si>
+  <si>
+    <t>بلدية الميلاد</t>
+  </si>
+  <si>
+    <t>اسم الاب</t>
+  </si>
+  <si>
+    <t>لقب الام</t>
+  </si>
+  <si>
+    <t>اسم الام</t>
+  </si>
+  <si>
+    <t>اسم الزوج(ة)</t>
+  </si>
+  <si>
+    <t>لقب الزوج(ة)</t>
+  </si>
+  <si>
+    <t>تاريخ ميلاد الزوج(ة)</t>
+  </si>
+  <si>
+    <t>رقم عقد ميلاد الزوج(ة)</t>
+  </si>
+  <si>
+    <t>بلدية ميلاد الزوج(ة)</t>
+  </si>
+  <si>
+    <t>اسم أب الزوج(ة)</t>
+  </si>
+  <si>
+    <t>اسم أم الزوج(ة)</t>
+  </si>
+  <si>
+    <t>لقب أم الزوج(ة)</t>
+  </si>
+  <si>
+    <t>الملاحظة</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -241,20 +192,6 @@
       <b/>
       <sz val="20"/>
       <color rgb="FF008000"/>
-      <name val="Mohammad Bold Normal"/>
-      <charset val="178"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color indexed="10"/>
-      <name val="Mohammad Bold Normal"/>
-      <charset val="178"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color indexed="8"/>
       <name val="Mohammad Bold Normal"/>
       <charset val="178"/>
     </font>
@@ -367,7 +304,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyFont="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyFont="0">
       <alignment horizontal="center"/>
@@ -375,7 +312,7 @@
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -394,33 +331,33 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="12">
-    <cellStyle name="Currency" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="Currency 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Currency" xfId="5"/>
+    <cellStyle name="Currency 2" xfId="9"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 2 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Normal 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Normal 2 4" xfId="10" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Normal 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Style 1" xfId="2" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="Style 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Style 2 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Style 6" xfId="4" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="Normal 2" xfId="6"/>
+    <cellStyle name="Normal 2 2" xfId="7"/>
+    <cellStyle name="Normal 2 3" xfId="1"/>
+    <cellStyle name="Normal 2 4" xfId="10"/>
+    <cellStyle name="Normal 3" xfId="3"/>
+    <cellStyle name="Style 1" xfId="2"/>
+    <cellStyle name="Style 2" xfId="8"/>
+    <cellStyle name="Style 2 2" xfId="11"/>
+    <cellStyle name="Style 6" xfId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -697,7 +634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AG15"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -739,100 +676,100 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="M1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="R1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="W1" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="AA1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="AE1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="AF1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="AG1" s="11" t="s">
         <v>31</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="U1" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="V1" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="W1" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="X1" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="AB1" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC1" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="AF1" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="AG1" s="11" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:33" s="12" customFormat="1" ht="27.75" thickTop="1" thickBot="1">
@@ -1326,8 +1263,8 @@
       <c r="AG15" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG1" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AE86">
+  <autoFilter ref="A1:AG1">
+    <sortState ref="A2:AE86">
       <sortCondition ref="C1"/>
     </sortState>
   </autoFilter>

</xml_diff>